<commit_message>
Repository unit tests updated
</commit_message>
<xml_diff>
--- a/documentation/Teszt_dokumentacio.xlsx
+++ b/documentation/Teszt_dokumentacio.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27932"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F79A4CA0-2771-4792-9D25-C9DE406CA2D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{305623B9-CFC7-47AA-B3FE-B5EAD0E353F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="22">
   <si>
     <t>ID</t>
   </si>
@@ -120,15 +120,6 @@
   </si>
   <si>
     <t>pass</t>
-  </si>
-  <si>
-    <t>Task2</t>
-  </si>
-  <si>
-    <t>fail</t>
-  </si>
-  <si>
-    <t>Task3</t>
   </si>
 </sst>
 </file>
@@ -270,7 +261,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -346,6 +337,10 @@
     <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="15" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="15" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normál" xfId="0" builtinId="0"/>
@@ -792,7 +787,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{099ACA43-BC8E-4EEF-8E46-10110C9E34F2}">
-  <dimension ref="A1:I8"/>
+  <dimension ref="A1:I14"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="15.77734375" customWidth="1"/>
@@ -855,82 +850,30 @@
         <v>PASS</v>
       </c>
       <c r="H2" s="25"/>
-      <c r="I2" s="26" t="str">
+      <c r="I2" s="27" t="str">
         <f ca="1">TEXT(TODAY(),"éééé.hh.nn.")</f>
         <v>2025.12.03.</v>
       </c>
     </row>
-    <row r="3" spans="1:9" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="21">
-        <v>2</v>
-      </c>
-      <c r="B3" s="21" t="s">
-        <v>22</v>
-      </c>
-      <c r="C3" s="22" t="s">
-        <v>19</v>
-      </c>
-      <c r="D3" s="23" t="s">
-        <v>20</v>
-      </c>
-      <c r="E3" s="23" t="s">
-        <v>21</v>
-      </c>
-      <c r="F3" s="23" t="s">
-        <v>23</v>
-      </c>
-      <c r="G3" s="24" t="str">
-        <f t="shared" ref="G3:G4" si="0">IF(TRIM(H3)&lt;&gt;"","On-Hold",IF(E3=F3,"PASS","FAIL"))</f>
-        <v>FAIL</v>
-      </c>
-      <c r="H3" s="25"/>
-      <c r="I3" s="26" t="str">
-        <f ca="1">TEXT(TODAY(),"éééé.hh.nn.")</f>
-        <v>2025.12.03.</v>
-      </c>
-    </row>
-    <row r="4" spans="1:9" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="21">
-        <v>3</v>
-      </c>
-      <c r="B4" s="21" t="s">
-        <v>24</v>
-      </c>
-      <c r="C4" s="22" t="s">
-        <v>19</v>
-      </c>
-      <c r="D4" s="23" t="s">
-        <v>20</v>
-      </c>
-      <c r="E4" s="23" t="s">
-        <v>23</v>
-      </c>
-      <c r="F4" s="23" t="s">
-        <v>23</v>
-      </c>
-      <c r="G4" s="24" t="str">
-        <f t="shared" si="0"/>
-        <v>PASS</v>
-      </c>
-      <c r="H4" s="25"/>
-      <c r="I4" s="26" t="str">
-        <f ca="1">TEXT(TODAY(),"éééé.hh.nn.")</f>
-        <v>2025.12.03.</v>
-      </c>
-    </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="I8" s="15"/>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="I6" s="15"/>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="G10" s="28"/>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="E14" s="28"/>
     </row>
   </sheetData>
   <phoneticPr fontId="5" type="noConversion"/>
-  <conditionalFormatting sqref="G2:G4">
-    <cfRule type="expression" dxfId="5" priority="1">
+  <conditionalFormatting sqref="G2">
+    <cfRule type="expression" dxfId="2" priority="1">
       <formula>TRIM($H2)&lt;&gt;""</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="4" priority="2">
+    <cfRule type="expression" dxfId="1" priority="2">
       <formula>$E2&lt;&gt;$F2</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="3" priority="3">
+    <cfRule type="expression" dxfId="0" priority="3">
       <formula>$E2=$F2</formula>
     </cfRule>
   </conditionalFormatting>
@@ -941,7 +884,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E9E478B6-D4CC-48C0-BEFA-B32A60FF6467}">
-  <dimension ref="A1:I4"/>
+  <dimension ref="A1:I2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="15.77734375" customWidth="1"/>
@@ -1009,74 +952,16 @@
         <v>2025.12.03.</v>
       </c>
     </row>
-    <row r="3" spans="1:9" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="21">
-        <v>2</v>
-      </c>
-      <c r="B3" s="21" t="s">
-        <v>22</v>
-      </c>
-      <c r="C3" s="22" t="s">
-        <v>19</v>
-      </c>
-      <c r="D3" s="23" t="s">
-        <v>20</v>
-      </c>
-      <c r="E3" s="23" t="s">
-        <v>21</v>
-      </c>
-      <c r="F3" s="23" t="s">
-        <v>23</v>
-      </c>
-      <c r="G3" s="24" t="str">
-        <f t="shared" ref="G3:G4" si="0">IF(TRIM(H3)&lt;&gt;"","On-Hold",IF(E3=F3,"PASS","FAIL"))</f>
-        <v>FAIL</v>
-      </c>
-      <c r="H3" s="25"/>
-      <c r="I3" s="26" t="str">
-        <f ca="1">TEXT(TODAY(),"éééé.hh.nn.")</f>
-        <v>2025.12.03.</v>
-      </c>
-    </row>
-    <row r="4" spans="1:9" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="21">
-        <v>3</v>
-      </c>
-      <c r="B4" s="21" t="s">
-        <v>24</v>
-      </c>
-      <c r="C4" s="22" t="s">
-        <v>19</v>
-      </c>
-      <c r="D4" s="23" t="s">
-        <v>20</v>
-      </c>
-      <c r="E4" s="23" t="s">
-        <v>23</v>
-      </c>
-      <c r="F4" s="23" t="s">
-        <v>23</v>
-      </c>
-      <c r="G4" s="24" t="str">
-        <f t="shared" si="0"/>
-        <v>PASS</v>
-      </c>
-      <c r="H4" s="25"/>
-      <c r="I4" s="26" t="str">
-        <f ca="1">TEXT(TODAY(),"éééé.hh.nn.")</f>
-        <v>2025.12.03.</v>
-      </c>
-    </row>
   </sheetData>
   <phoneticPr fontId="5" type="noConversion"/>
-  <conditionalFormatting sqref="G2:G4">
-    <cfRule type="expression" dxfId="2" priority="1">
+  <conditionalFormatting sqref="G2">
+    <cfRule type="expression" dxfId="5" priority="1">
       <formula>TRIM($H2)&lt;&gt;""</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="1" priority="2">
+    <cfRule type="expression" dxfId="4" priority="2">
       <formula>$E2&lt;&gt;$F2</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="0" priority="3">
+    <cfRule type="expression" dxfId="3" priority="3">
       <formula>$E2=$F2</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>